<commit_message>
Added some additional caveats about unmarked smelt
</commit_message>
<xml_diff>
--- a/Running Delta Smelt Catch.xlsx
+++ b/Running Delta Smelt Catch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cawater-my.sharepoint.com/personal/rosemary_hartman_water_ca_gov/Documents/smelt cages/SmeltMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="99" documentId="13_ncr:1_{F25AE125-BFC2-4782-A524-81D3BA29BCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61547D95-C0F5-4A56-B775-6608916F00CF}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="13_ncr:1_{F25AE125-BFC2-4782-A524-81D3BA29BCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9B313CB-CA51-4D67-9DEB-45BC3709C04C}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{4BB403AD-DB3F-4CB5-B7F1-39827ED458E8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{4BB403AD-DB3F-4CB5-B7F1-39827ED458E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="12" r:id="rId1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5858" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6011" uniqueCount="735">
   <si>
     <t>Running Delta Smelt Catch Data Collected for the USFWS Delta Smelt Experimental Release Technical Team</t>
   </si>
@@ -2277,6 +2277,39 @@
   <si>
     <t>26-17-SM03</t>
   </si>
+  <si>
+    <t>26-19-SM01</t>
+  </si>
+  <si>
+    <t>26-19-SSC01</t>
+  </si>
+  <si>
+    <t>26-20-SM01</t>
+  </si>
+  <si>
+    <t>26-20-SM05</t>
+  </si>
+  <si>
+    <t>unknown</t>
+  </si>
+  <si>
+    <t>26-20-SM06</t>
+  </si>
+  <si>
+    <t>26-20-SM02</t>
+  </si>
+  <si>
+    <t>26-21-SM05</t>
+  </si>
+  <si>
+    <t>26-21-SM04</t>
+  </si>
+  <si>
+    <t>26-22-SM03</t>
+  </si>
+  <si>
+    <t>26-22-SM02</t>
+  </si>
 </sst>
 </file>
 
@@ -2285,7 +2318,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2392,6 +2425,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -2459,7 +2498,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2614,6 +2653,8 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3342,7 +3383,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C569B310-60E0-4E31-89EB-52CC1C810311}">
-  <dimension ref="A1:AT412"/>
+  <dimension ref="A1:AT426"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.26953125" bestFit="1" customWidth="1"/>
@@ -32756,6 +32797,790 @@
         <v>638</v>
       </c>
     </row>
+    <row r="413" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A413" t="s">
+        <v>87</v>
+      </c>
+      <c r="B413" s="25">
+        <v>45992</v>
+      </c>
+      <c r="C413" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D413" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E413" t="s">
+        <v>724</v>
+      </c>
+      <c r="F413" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G413">
+        <v>14708</v>
+      </c>
+      <c r="H413">
+        <v>11.8999996185303</v>
+      </c>
+      <c r="J413">
+        <v>32.849998474121101</v>
+      </c>
+      <c r="K413" s="10">
+        <v>66</v>
+      </c>
+      <c r="L413" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M413" s="64">
+        <v>38.170079999999999</v>
+      </c>
+      <c r="N413" s="64">
+        <v>-122.02123</v>
+      </c>
+      <c r="S413" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T413" s="10" t="s">
+        <v>721</v>
+      </c>
+      <c r="U413" s="25">
+        <v>45965</v>
+      </c>
+      <c r="V413" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W413" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="414" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A414" t="s">
+        <v>87</v>
+      </c>
+      <c r="B414" s="25">
+        <v>45995</v>
+      </c>
+      <c r="C414" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D414" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E414" t="s">
+        <v>725</v>
+      </c>
+      <c r="F414" t="s">
+        <v>108</v>
+      </c>
+      <c r="G414">
+        <v>485.70001220703102</v>
+      </c>
+      <c r="H414">
+        <v>12.300000190734901</v>
+      </c>
+      <c r="J414">
+        <v>47.310001373291001</v>
+      </c>
+      <c r="K414">
+        <v>73</v>
+      </c>
+      <c r="L414" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M414" s="62">
+        <v>38.4163</v>
+      </c>
+      <c r="N414" s="62">
+        <v>-121.61008</v>
+      </c>
+      <c r="S414" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="T414" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="U414" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="V414" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="W414" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="415" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A415" t="s">
+        <v>87</v>
+      </c>
+      <c r="B415" s="65">
+        <v>46000</v>
+      </c>
+      <c r="C415" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D415" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E415" t="s">
+        <v>726</v>
+      </c>
+      <c r="F415" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G415">
+        <v>9337</v>
+      </c>
+      <c r="H415">
+        <v>9.8999996185302699</v>
+      </c>
+      <c r="J415">
+        <v>19.940000534057599</v>
+      </c>
+      <c r="K415">
+        <v>74</v>
+      </c>
+      <c r="L415" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M415" s="62">
+        <v>38.185200000000002</v>
+      </c>
+      <c r="N415" s="62">
+        <v>-121.96747999999999</v>
+      </c>
+      <c r="S415" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T415" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U415" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V415" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W415" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="416" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A416" t="s">
+        <v>87</v>
+      </c>
+      <c r="B416" s="65">
+        <v>46000</v>
+      </c>
+      <c r="C416" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D416" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E416" t="s">
+        <v>726</v>
+      </c>
+      <c r="F416" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G416">
+        <v>9288</v>
+      </c>
+      <c r="H416">
+        <v>9.8999996185302699</v>
+      </c>
+      <c r="J416">
+        <v>14.5</v>
+      </c>
+      <c r="K416">
+        <v>69</v>
+      </c>
+      <c r="L416" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M416" s="62">
+        <v>38.185090000000002</v>
+      </c>
+      <c r="N416" s="62">
+        <v>-121.96746</v>
+      </c>
+      <c r="S416" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T416" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U416" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V416" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W416" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="417" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A417" t="s">
+        <v>87</v>
+      </c>
+      <c r="B417" s="65">
+        <v>46000</v>
+      </c>
+      <c r="C417" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D417" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E417" t="s">
+        <v>727</v>
+      </c>
+      <c r="F417" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G417">
+        <v>8959</v>
+      </c>
+      <c r="H417">
+        <v>10.1000003814697</v>
+      </c>
+      <c r="J417">
+        <v>20.610000610351602</v>
+      </c>
+      <c r="K417">
+        <v>61</v>
+      </c>
+      <c r="L417" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M417" s="62">
+        <v>38.175350000000002</v>
+      </c>
+      <c r="N417" s="62">
+        <v>-121.94952000000001</v>
+      </c>
+      <c r="S417" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T417" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U417" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V417" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W417" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="418" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A418" t="s">
+        <v>87</v>
+      </c>
+      <c r="B418" s="65">
+        <v>46002</v>
+      </c>
+      <c r="C418" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D418" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E418" t="s">
+        <v>729</v>
+      </c>
+      <c r="F418" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G418">
+        <v>14940</v>
+      </c>
+      <c r="H418">
+        <v>9.8000001907348597</v>
+      </c>
+      <c r="J418">
+        <v>53.310001373291001</v>
+      </c>
+      <c r="K418">
+        <v>55</v>
+      </c>
+      <c r="L418" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M418" s="62">
+        <v>38.162849999999999</v>
+      </c>
+      <c r="N418" s="62">
+        <v>-122.0449</v>
+      </c>
+      <c r="S418" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T418" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U418" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V418" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W418" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="419" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A419" t="s">
+        <v>87</v>
+      </c>
+      <c r="B419" s="65">
+        <v>46002</v>
+      </c>
+      <c r="C419" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D419" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E419" t="s">
+        <v>729</v>
+      </c>
+      <c r="F419" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G419">
+        <v>14940</v>
+      </c>
+      <c r="H419">
+        <v>9.8000001907348597</v>
+      </c>
+      <c r="J419">
+        <v>53.310001373291001</v>
+      </c>
+      <c r="K419">
+        <v>56</v>
+      </c>
+      <c r="L419" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M419" s="62">
+        <v>38.162849999999999</v>
+      </c>
+      <c r="N419" s="62">
+        <v>-122.0449</v>
+      </c>
+      <c r="S419" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T419" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U419" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V419" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W419" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="420" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A420" t="s">
+        <v>87</v>
+      </c>
+      <c r="B420" s="65">
+        <v>46002</v>
+      </c>
+      <c r="C420" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D420" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E420" t="s">
+        <v>729</v>
+      </c>
+      <c r="F420" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G420">
+        <v>14940</v>
+      </c>
+      <c r="H420">
+        <v>9.8000001907348597</v>
+      </c>
+      <c r="J420">
+        <v>53.310001373291001</v>
+      </c>
+      <c r="K420">
+        <v>57</v>
+      </c>
+      <c r="L420" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M420" s="62">
+        <v>38.162849999999999</v>
+      </c>
+      <c r="N420" s="62">
+        <v>-122.0449</v>
+      </c>
+      <c r="S420" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T420" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U420" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V420" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W420" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="421" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A421" t="s">
+        <v>87</v>
+      </c>
+      <c r="B421" s="65">
+        <v>46002</v>
+      </c>
+      <c r="C421" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D421" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E421" t="s">
+        <v>729</v>
+      </c>
+      <c r="F421" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G421">
+        <v>14940</v>
+      </c>
+      <c r="H421">
+        <v>9.8000001907348597</v>
+      </c>
+      <c r="J421">
+        <v>53.310001373291001</v>
+      </c>
+      <c r="K421">
+        <v>70</v>
+      </c>
+      <c r="L421" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M421" s="62">
+        <v>38.162849999999999</v>
+      </c>
+      <c r="N421" s="62">
+        <v>-122.0449</v>
+      </c>
+      <c r="S421" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T421" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U421" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V421" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W421" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="422" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A422" t="s">
+        <v>87</v>
+      </c>
+      <c r="B422" s="65">
+        <v>46002</v>
+      </c>
+      <c r="C422" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D422" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E422" t="s">
+        <v>730</v>
+      </c>
+      <c r="F422" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G422">
+        <v>11186</v>
+      </c>
+      <c r="H422">
+        <v>9.3000001907348597</v>
+      </c>
+      <c r="J422">
+        <v>32.169998168945298</v>
+      </c>
+      <c r="K422">
+        <v>59</v>
+      </c>
+      <c r="L422" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M422" s="62">
+        <v>38.17895</v>
+      </c>
+      <c r="N422" s="62">
+        <v>-122.04688</v>
+      </c>
+      <c r="S422" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T422" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U422" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V422" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W422" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="423" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A423" t="s">
+        <v>87</v>
+      </c>
+      <c r="B423" s="63">
+        <v>46007</v>
+      </c>
+      <c r="C423" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D423" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E423" t="s">
+        <v>731</v>
+      </c>
+      <c r="F423" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G423">
+        <v>7259</v>
+      </c>
+      <c r="H423">
+        <v>9.3999996185302699</v>
+      </c>
+      <c r="J423">
+        <v>13.420000076293899</v>
+      </c>
+      <c r="K423">
+        <v>57</v>
+      </c>
+      <c r="L423" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M423" s="62">
+        <v>38.149149999999999</v>
+      </c>
+      <c r="N423" s="62">
+        <v>-121.91477999999999</v>
+      </c>
+      <c r="S423" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T423" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U423" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V423" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W423" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="424" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A424" t="s">
+        <v>87</v>
+      </c>
+      <c r="B424" s="63">
+        <v>46007</v>
+      </c>
+      <c r="C424" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D424" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E424" t="s">
+        <v>732</v>
+      </c>
+      <c r="F424" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G424">
+        <v>17143</v>
+      </c>
+      <c r="H424">
+        <v>9</v>
+      </c>
+      <c r="J424">
+        <v>20.7700004577637</v>
+      </c>
+      <c r="K424">
+        <v>47</v>
+      </c>
+      <c r="L424" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M424" s="62">
+        <v>38.160080000000001</v>
+      </c>
+      <c r="N424" s="62">
+        <v>-122.05856</v>
+      </c>
+      <c r="S424" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T424" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U424" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V424" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W424" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="425" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A425" t="s">
+        <v>87</v>
+      </c>
+      <c r="B425" s="65">
+        <v>46012</v>
+      </c>
+      <c r="C425" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D425" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E425" t="s">
+        <v>733</v>
+      </c>
+      <c r="F425" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G425">
+        <v>8588</v>
+      </c>
+      <c r="H425">
+        <v>11.1000003814697</v>
+      </c>
+      <c r="J425">
+        <v>11.920000076293899</v>
+      </c>
+      <c r="K425">
+        <v>54</v>
+      </c>
+      <c r="L425" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M425" s="62">
+        <v>38.171109999999999</v>
+      </c>
+      <c r="N425" s="62">
+        <v>-121.96088</v>
+      </c>
+      <c r="S425" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T425" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U425" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V425" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W425" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="426" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A426" t="s">
+        <v>87</v>
+      </c>
+      <c r="B426" s="65">
+        <v>46012</v>
+      </c>
+      <c r="C426" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D426" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E426" t="s">
+        <v>734</v>
+      </c>
+      <c r="F426" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="G426">
+        <v>15256</v>
+      </c>
+      <c r="H426">
+        <v>10.800000190734901</v>
+      </c>
+      <c r="J426">
+        <v>34.610000610351598</v>
+      </c>
+      <c r="K426">
+        <v>55</v>
+      </c>
+      <c r="L426" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="M426" s="62">
+        <v>38.168610000000001</v>
+      </c>
+      <c r="N426" s="62">
+        <v>-122.06841</v>
+      </c>
+      <c r="S426" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="T426" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="U426" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="V426" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="W426" s="48" t="s">
+        <v>638</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AT378">
     <sortCondition ref="B2:B378"/>
@@ -32965,15 +33790,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="65146633-a755-433a-aacb-5024b6511b89">
@@ -33004,6 +33820,15 @@
     </SharedWithUsers>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -33242,20 +34067,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7C764E5-19B4-4012-98BF-B46F2FA7A2CF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D4F8AF6-B64B-4962-81B5-D73EE7A1E0CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="65146633-a755-433a-aacb-5024b6511b89"/>
     <ds:schemaRef ds:uri="d8e23be6-d007-4c2c-9265-7d9405abf22e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7C764E5-19B4-4012-98BF-B46F2FA7A2CF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>